<commit_message>
docs(inputs): S16-01 questions Q-38 and Q-39 for OQ-38 and OQ-39 of spec 0.3.1
Added to the Questions sheet's XML only, so the cached values of the
formulas in the other sheets stay as Excel saved them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/BCS_inputs_v1_demo.xlsx
+++ b/docs/inputs/BCS_inputs_v1_demo.xlsx
@@ -9248,7 +9248,7 @@
     <tabColor rgb="FF1F4E78"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
@@ -10449,6 +10449,84 @@
       </c>
       <c r="H46" s="13"/>
       <c r="I46" s="12"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>Q-38</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>จัดซื้อ</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>คิวจัดซื้อถือว่าทันเวลาเมื่อส่ง PO ขออนุมัติภายในกี่ชั่วโมงทำการหลังคำขออนุมัติ</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>การ์ดงานอนุมัติทันเวลาบนหน้าแรก (§11.5)</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>16 ชั่วโมงทำการ (procurement.queueTargetBusinessMinutes = 960)</t>
+        </is>
+      </c>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>OQ-38</t>
+        </is>
+      </c>
+      <c r="H47" s="13"/>
+      <c r="I47" s="13"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t>Q-39</t>
+        </is>
+      </c>
+      <c r="B48" s="12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>CEO COO</t>
+        </is>
+      </c>
+      <c r="D48" s="12" t="inlineStr">
+        <is>
+          <t>ผู้ขอเพิ่มคนที่ยังไม่เห็นคำขอเป็นผู้ติดตามได้หรือไม่ (ถ้าได้ ผู้ถูกเพิ่มจะเห็นใบเสนอราคาและไฟล์แนบของคำขอนั้น)</t>
+        </is>
+      </c>
+      <c r="E48" s="12" t="inlineStr">
+        <is>
+          <t>สิทธิ์ดูคำขอและไฟล์แนบ</t>
+        </is>
+      </c>
+      <c r="F48" s="12" t="inlineStr">
+        <is>
+          <t>ไม่ได้ · เพิ่มได้เฉพาะสมาชิกที่เห็นคำขออยู่แล้ว การติดตามไม่ขยายสิทธิ์ดู</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>OQ-39</t>
+        </is>
+      </c>
+      <c r="H48" s="13"/>
+      <c r="I48" s="13"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>